<commit_message>
WIP: working on truck layout
</commit_message>
<xml_diff>
--- a/public/Program do szacowania kosztów transportu.xlsx
+++ b/public/Program do szacowania kosztów transportu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\OneDrive\Pulpit\Angular\transport-cost-estimator\transport-cost-estimator\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D80E808A-E81A-42E1-B3E1-A48332E10AD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0BECD6C-A1A4-47B7-9562-0EFB0CC5E99A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57495" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="40230" yWindow="1830" windowWidth="28800" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -417,7 +417,7 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>